<commit_message>
fix ablation eval to include scenes 29-34 in per-scene sheets
</commit_message>
<xml_diff>
--- a/data/analysis_ministral_3_14b_panns/multimodal_event_eval_ministral_3_14b_panns_w2_5s_h1_25s.xlsx
+++ b/data/analysis_ministral_3_14b_panns/multimodal_event_eval_ministral_3_14b_panns_w2_5s_h1_25s.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="52">
   <si>
     <t>event</t>
   </si>
@@ -103,39 +103,36 @@
     <t>YES</t>
   </si>
   <si>
-    <t>fight(48-144)</t>
-  </si>
-  <si>
-    <t>fight(96-168)</t>
-  </si>
-  <si>
-    <t>fight(72-72)</t>
-  </si>
-  <si>
-    <t>gunshot_or_explosion(90-240)</t>
+    <t>sound: engine(150-210), visual: physical_altercation(48-96), visual: physical_altercation(72-144), visual: physical_altercation(48-48), visual: physical_altercation(144-144), visual: running(48-192), visual: running(96-216)</t>
+  </si>
+  <si>
+    <t>visual: carrying(72-144), visual: physical_altercation(96-144), visual: physical_altercation(168-168), visual: running(72-168), visual: running(192-216), visual: running(192-216), visual: suspicious_near_vehicle(0-0), visual: suspicious_near_vehicle(192-216), visual: suspicious_near_vehicle(0-0), visual: suspicious_near_vehicle(24-120), visual: suspicious_near_vehicle(96-96), visual: suspicious_near_vehicle(168-168)</t>
+  </si>
+  <si>
+    <t>sound: engine(180-240), visual: carrying(120-120), visual: physical_altercation(72-72)</t>
   </si>
   <si>
     <t>sound: gunshot_or_explosion(90-180), sound: engine(150-240), visual: explosion_visible(120-120), visual: explosion_visible(144-240), visual: gunshot_visible(168-168), visual: running(120-240), visual: suspicious_near_vehicle(0-0), visual: suspicious_near_vehicle(24-24), visual: suspicious_near_vehicle(0-0), visual: suspicious_near_vehicle(24-120), visual: vehicle_collision(216-240)</t>
   </si>
   <si>
-    <t>gunshot_or_explosion(30-120)</t>
-  </si>
-  <si>
-    <t>gunshot_or_explosion(120-180)</t>
-  </si>
-  <si>
-    <t>gunshot_or_explosion(0-240)</t>
+    <t>sound: engine(0-60), sound: gunshot_or_explosion(30-120), visual: enter_or_exit_vehicle(0-0), visual: enter_or_exit_vehicle(72-72), visual: enter_or_exit_vehicle(144-144), visual: enter_or_exit_vehicle(120-120), visual: enter_or_exit_vehicle(0-0), visual: enter_or_exit_vehicle(48-72), visual: suspicious_near_vehicle(0-0), visual: suspicious_near_vehicle(96-120), visual: suspicious_near_vehicle(48-72), visual: suspicious_near_vehicle(144-144), visual: suspicious_near_vehicle(0-0), visual: suspicious_near_vehicle(0-0), visual: suspicious_near_vehicle(0-0), visual: suspicious_near_vehicle(0-0), visual: suspicious_near_vehicle(0-0), visual: suspicious_near_vehicle(0-0), visual: suspicious_near_vehicle(48-144), visual: suspicious_near_vehicle(0-0)</t>
+  </si>
+  <si>
+    <t>sound: engine(0-60), sound: engine(150-240), sound: gunshot_or_explosion(120-180), visual: carrying(144-216), visual: enter_or_exit_vehicle(48-48), visual: enter_or_exit_vehicle(96-96), visual: enter_or_exit_vehicle(96-96), visual: explosion_visible(120-120), visual: gunshot_visible(120-120), visual: running(144-144), visual: running(120-120), visual: suspicious_near_vehicle(24-24), visual: suspicious_near_vehicle(216-216), visual: suspicious_near_vehicle(48-48), visual: suspicious_near_vehicle(144-168), visual: suspicious_near_vehicle(96-120), visual: suspicious_near_vehicle(192-192), visual: suspicious_near_vehicle(216-216), visual: suspicious_near_vehicle(168-192), visual: suspicious_near_vehicle(168-216), visual: suspicious_near_vehicle(144-144), visual: suspicious_near_vehicle(96-96)</t>
+  </si>
+  <si>
+    <t>sound: gunshot_or_explosion(0-90), sound: engine(60-120), sound: engine(180-240), visual: explosion_visible(24-240), visual: running(24-240), visual: running(120-240)</t>
   </si>
   <si>
     <t>sound: gunshot_or_explosion(0-90), sound: engine(120-240), visual: enter_or_exit_vehicle(0-0), visual: explosion_visible(72-72), visual: explosion_visible(144-240), visual: explosion_visible(216-240), visual: explosion_visible(72-72), visual: explosion_visible(216-240), visual: explosion_visible(48-216), visual: explosion_visible(168-168), visual: running(96-240), visual: suspicious_near_vehicle(24-24), visual: suspicious_near_vehicle(0-0), visual: suspicious_near_vehicle(216-240), visual: suspicious_near_vehicle(216-240), visual: suspicious_near_vehicle(0-24), visual: suspicious_near_vehicle(96-96), visual: suspicious_near_vehicle(216-240), visual: vehicle_collision(48-240), visual: vehicle_collision(48-48), visual: vehicle_collision(192-240), visual: vehicle_collision(72-120), visual: vehicle_collision(216-240)</t>
   </si>
   <si>
-    <t>vehicle_escape(24-48)</t>
-  </si>
-  <si>
     <t>sound: engine(60-240), visual: carrying(120-240), visual: carrying(72-96), visual: carrying(168-216), visual: carrying(24-48), visual: carrying(144-240), visual: enter_or_exit_vehicle(120-240), visual: enter_or_exit_vehicle(48-48), visual: enter_or_exit_vehicle(240-240), visual: running(24-24), visual: suspicious_near_vehicle(72-240), visual: suspicious_near_vehicle(24-48), visual: suspicious_near_vehicle(120-240)</t>
   </si>
   <si>
+    <t>visual: carrying(120-240), visual: carrying(72-96), visual: carrying(168-216), visual: carrying(24-48), visual: carrying(144-240), visual: enter_or_exit_vehicle(120-240), visual: enter_or_exit_vehicle(48-48), visual: enter_or_exit_vehicle(240-240), visual: running(24-24), visual: suspicious_near_vehicle(72-240), visual: suspicious_near_vehicle(24-48), visual: suspicious_near_vehicle(120-240)</t>
+  </si>
+  <si>
     <t>NO</t>
   </si>
   <si>
@@ -148,70 +145,61 @@
     <t>sound: horn(0-90), sound: engine(120-210), visual: enter_or_exit_vehicle(192-192), visual: suspicious_near_vehicle(192-192)</t>
   </si>
   <si>
-    <t>vehicle_collision(30-240)</t>
-  </si>
-  <si>
     <t>sound: engine(0-60), sound: skidding(30-90), sound: gunshot_or_explosion(60-120), sound: glass_breaking(90-150), visual: 9(240-240), visual: enter_or_exit_vehicle(168-168), visual: enter_or_exit_vehicle(240-240), visual: suspicious_near_vehicle(240-240), visual: suspicious_near_vehicle(72-168), visual: suspicious_near_vehicle(72-144), visual: suspicious_near_vehicle(192-240), visual: vehicle_collision(72-240), visual: vehicle_collision(96-240), visual: vehicle_collision(72-72)</t>
   </si>
   <si>
-    <t>vehicle_collision(120-240)</t>
-  </si>
-  <si>
     <t>sound: horn(0-60), sound: engine(30-240), sound: gunshot_or_explosion(60-120), visual: 9(120-120), visual: enter_or_exit_vehicle(120-120), visual: enter_or_exit_vehicle(144-144), visual: enter_or_exit_vehicle(216-240), visual: enter_or_exit_vehicle(168-192), visual: enter_or_exit_vehicle(168-240), visual: suspicious_near_vehicle(216-240), visual: suspicious_near_vehicle(168-192), visual: suspicious_near_vehicle(168-240), visual: vehicle_collision(120-144), visual: vehicle_collision(216-240), visual: vehicle_collision(168-192)</t>
   </si>
   <si>
-    <t>loitering(24-216)</t>
-  </si>
-  <si>
-    <t>loitering(0-192)</t>
+    <t>visual: enter_or_exit_vehicle(24-48), visual: suspicious_near_vehicle(24-216), visual: suspicious_near_vehicle(240-240)</t>
+  </si>
+  <si>
+    <t>visual: running(216-216), visual: suspicious_near_vehicle(24-216)</t>
   </si>
   <si>
     <t>visual: carrying(192-240), visual: enter_or_exit_vehicle(96-168), visual: enter_or_exit_vehicle(192-240), visual: running(72-72), visual: suspicious_near_vehicle(0-192), visual: suspicious_near_vehicle(216-240), visual: suspicious_near_vehicle(192-192)</t>
   </si>
   <si>
-    <t>handoff(24-192), handoff(24-192)</t>
-  </si>
-  <si>
-    <t>handoff(72-240), handoff(168-240), handoff(24-120), handoff(0-192), handoff(144-192), handoff(72-240), handoff(168-240), handoff(24-120), handoff(0-192), handoff(144-192)</t>
-  </si>
-  <si>
-    <t>handoff(48-96), handoff(24-72), handoff(96-192), handoff(24-192), handoff(0-72), handoff(0-192), handoff(48-96), handoff(96-192), handoff(48-96), handoff(96-192), handoff(24-96), handoff(0-72), handoff(48-96), handoff(0-192), handoff(96-192), handoff(24-72), handoff(24-192), handoff(24-96)</t>
+    <t>visual: carrying(0-0), visual: carrying(24-144), visual: carrying(144-144), visual: carrying(168-192)</t>
+  </si>
+  <si>
+    <t>visual: carrying(24-24), visual: carrying(192-240), visual: carrying(96-120), visual: carrying(0-0), visual: carrying(144-168), visual: carrying(216-216), visual: carrying(120-144), visual: carrying(72-72), visual: carrying(168-168), visual: carrying(240-240), visual: carrying(24-48), visual: carrying(192-192), visual: suspicious_near_vehicle(240-240), visual: suspicious_near_vehicle(240-240)</t>
+  </si>
+  <si>
+    <t>visual: carrying(48-72), visual: carrying(192-192), visual: carrying(0-24), visual: carrying(96-96), visual: carrying(96-96), visual: carrying(48-72), visual: carrying(144-192), visual: carrying(120-120), visual: carrying(24-24), visual: carrying(144-192), visual: suspicious_near_vehicle(96-96), visual: suspicious_near_vehicle(192-192), visual: suspicious_near_vehicle(48-72), visual: suspicious_near_vehicle(96-168), visual: suspicious_near_vehicle(0-0), visual: suspicious_near_vehicle(0-0), visual: suspicious_near_vehicle(48-72), visual: suspicious_near_vehicle(144-168)</t>
   </si>
   <si>
     <t>visual: physical_altercation(48-120)</t>
   </si>
   <si>
-    <t>fight(48-120)</t>
-  </si>
-  <si>
-    <t>vehicle_escape(24-72)</t>
-  </si>
-  <si>
-    <t>vehicle_escape(0-240)</t>
+    <t>visual: physical_altercation(48-120), visual: running(24-120), visual: running(24-120), visual: running(192-192), visual: running(192-192)</t>
+  </si>
+  <si>
+    <t>sound: engine(90-240), visual: carrying(0-0), visual: carrying(24-48), visual: enter_or_exit_vehicle(72-72), visual: running(24-24), visual: suspicious_near_vehicle(0-72)</t>
   </si>
   <si>
     <t>sound: engine(60-240), visual: enter_or_exit_vehicle(48-240), visual: running(0-0), visual: suspicious_near_vehicle(0-192)</t>
   </si>
   <si>
-    <t>vehicle_collision(72-240)</t>
-  </si>
-  <si>
-    <t>vehicle_collision(48-240)</t>
-  </si>
-  <si>
-    <t>loitering(0-216)</t>
-  </si>
-  <si>
-    <t>loitering(24-240)</t>
+    <t>visual: enter_or_exit_vehicle(48-240), visual: running(0-0), visual: suspicious_near_vehicle(0-192)</t>
+  </si>
+  <si>
+    <t>sound: horn(0-90), sound: engine(120-210), visual: enter_or_exit_vehicle(168-240), visual: enter_or_exit_vehicle(192-216), visual: suspicious_near_vehicle(168-240), visual: suspicious_near_vehicle(192-216), visual: vehicle_collision(72-240), visual: vehicle_collision(72-240)</t>
+  </si>
+  <si>
+    <t>sound: skidding(0-90), visual: enter_or_exit_vehicle(168-168), visual: enter_or_exit_vehicle(240-240), visual: suspicious_near_vehicle(168-240), visual: vehicle_collision(48-240), visual: vehicle_collision(96-240), visual: vehicle_collision(48-72)</t>
+  </si>
+  <si>
+    <t>visual: carrying(0-0), visual: enter_or_exit_vehicle(72-168), visual: running(216-216), visual: suspicious_near_vehicle(0-216)</t>
   </si>
   <si>
     <t>visual: enter_or_exit_vehicle(48-168), visual: running(48-48), visual: running(192-240), visual: suspicious_near_vehicle(24-240)</t>
   </si>
   <si>
-    <t>handoff(0-216), handoff(0-216)</t>
-  </si>
-  <si>
-    <t>handoff(24-216), handoff(24-216)</t>
+    <t>visual: carrying(0-96), visual: carrying(120-120), visual: carrying(192-216), visual: carrying(48-48), visual: carrying(144-144)</t>
+  </si>
+  <si>
+    <t>visual: carrying(24-216), visual: carrying(168-168)</t>
   </si>
 </sst>
 </file>
@@ -795,7 +783,7 @@
         <v>4</v>
       </c>
       <c r="E2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -812,15 +800,59 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
         <v>29</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -844,13 +876,13 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>30</v>
+      <c r="C2" t="s">
+        <v>29</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
@@ -864,7 +896,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -888,13 +920,13 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>30</v>
+        <v>15</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>29</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
@@ -908,87 +940,43 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>15</v>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>16</v>
       </c>
       <c r="B2" t="s">
         <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
       </c>
       <c r="E2" t="s">
         <v>33</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>16</v>
-      </c>
-      <c r="B2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1005,7 +993,7 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1049,7 +1037,7 @@
         <v>4</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1066,139 +1054,139 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
         <v>37</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>18</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>19</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>20</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1215,6 +1203,182 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>21</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
         <v>40</v>
       </c>
     </row>
@@ -1223,7 +1387,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1247,16 +1411,16 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2">
-        <v>21</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
+        <v>29</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
       </c>
       <c r="E2" t="s">
         <v>41</v>
@@ -1267,7 +1431,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1291,7 +1455,7 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s">
         <v>8</v>
@@ -1303,15 +1467,15 @@
         <v>4</v>
       </c>
       <c r="E2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1335,54 +1499,10 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2">
-        <v>22</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>42</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>23</v>
-      </c>
-      <c r="B2" t="s">
-        <v>10</v>
+        <v>31</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
       </c>
       <c r="C2" t="s">
         <v>18</v>
@@ -1399,175 +1519,43 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>29</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
       </c>
       <c r="E2" t="s">
         <v>44</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>30</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>31</v>
-      </c>
-      <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>32</v>
-      </c>
-      <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1584,6 +1572,138 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>33</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>35</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1592,34 +1712,34 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>33</v>
-      </c>
-      <c r="B2" t="s">
-        <v>12</v>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>36</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
       </c>
       <c r="C2" t="s">
         <v>18</v>
@@ -1629,138 +1749,6 @@
       </c>
       <c r="E2" t="s">
         <v>49</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>34</v>
-      </c>
-      <c r="B2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>35</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>36</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1777,7 +1765,7 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1865,7 +1853,7 @@
         <v>4</v>
       </c>
       <c r="E2" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1909,7 +1897,7 @@
         <v>4</v>
       </c>
       <c r="E2" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -2014,6 +2002,50 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -2022,7 +2054,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2046,11 +2078,11 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2">
-        <v>8</v>
-      </c>
-      <c r="B2" t="s">
         <v>9</v>
       </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
       <c r="C2" t="s">
         <v>18</v>
       </c>
@@ -2066,7 +2098,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2090,11 +2122,11 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
       <c r="C2" t="s">
         <v>18</v>
       </c>
@@ -2103,50 +2135,6 @@
       </c>
       <c r="E2" t="s">
         <v>25</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -2207,7 +2195,7 @@
         <v>5</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>